<commit_message>
Set KRUE 220 kV serial numbers in the equipment summary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQNKmDw1ASSgZrXBD8UV4E
</commit_message>
<xml_diff>
--- a/Свод_оборудование_ГПП_РД_зав_номера_АоРПИ_v3.xlsx
+++ b/Свод_оборудование_ГПП_РД_зав_номера_АоРПИ_v3.xlsx
@@ -1333,7 +1333,7 @@
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>КРУЭ 220 кВ: зав. № SGF24012NSD01–04 только в отклонённом RFI 1440, АоРПИ нет; присланные 22.09.2026 документы (TP-0007) — только на ОПН. ТРДН — ОК (477/478). ОПН — 12 зав. № подтверждены паспортами TP-0007 1B, АоРПИ 1248 не подписан и без номеров. ШМУ, токопроводы, ШУ-Д — номеров нет.</t>
+          <t>КРУЭ 220 кВ: зав. № 22247473, 22247474, 22247492–22247495 (6 шт, внесены 28.09.2026); RFI 1440 отклонён, АоРПИ нет; присланные 22.09.2026 документы (TP-0007) — только на ОПН. ТРДН — ОК (477/478). ОПН — 12 зав. № подтверждены паспортами TP-0007 1B, АоРПИ 1248 не подписан и без номеров. ШМУ, токопроводы, ШУ-Д — номеров нет.</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="42" customHeight="1" s="19">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -11921,6 +11920,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="42" customHeight="1" s="19">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -27522,15 +27522,15 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>SGF24012NSD01; SGF24012NSD02; SGF24012NSD03; SGF24012NSD04</t>
+          <t>22247473; 22247474; 22247492; 22247493; 22247494; 22247495</t>
         </is>
       </c>
       <c r="G6" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>RFI 1440 (отклонён)</t>
+          <t>Данные пользователя (28.09.2026)</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -27554,7 +27554,7 @@
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>4 зав. № — по транспортным блокам КРУЭ. Документы Чэнда по RFI 1440 от 22.09.2026 (TRM 18712) — только паспорта ОПН (TP-0007), паспортов КРУЭ с зав. № нет. RFI 1440 отклонён, повторного RFI нет; АоРПИ нет</t>
+          <t>6 зав. № КРУЭ (22247473, 22247474, 22247492–22247495) внесены 28.09.2026 по данным пользователя. В отклонённом RFI 1440 были указаны зав. № транспортных блоков SGF24012NSD01–04. RFI 1440 отклонён, повторного RFI нет; АоРПИ нет</t>
         </is>
       </c>
       <c r="N6" s="6" t="n"/>

</xml_diff>